<commit_message>
Sync working files: updated config, remove stale runtime artifacts
</commit_message>
<xml_diff>
--- a/Client_Mapping_Sheet.xlsx
+++ b/Client_Mapping_Sheet.xlsx
@@ -413,8 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col hidden="1" width="16" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -444,7 +449,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>T#114-PE-C1C5-P0101</t>
+          <t>225-QF-D2D6-Q1212</t>
         </is>
       </c>
     </row>
@@ -459,7 +464,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>T#114-PE-C1C5-P0102</t>
+          <t>225-QF-D2D6-Q1213</t>
         </is>
       </c>
     </row>
@@ -469,12 +474,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>114-PG-C1C5-P0103</t>
+          <t>114-PE-C1C5-X060</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>T#114-PG-C1C5-P0103</t>
+          <t>225-QF-D2D6-Y171</t>
         </is>
       </c>
     </row>
@@ -484,12 +489,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>114GA-C1-C5#</t>
+          <t>114-PG-C1C5-P0103</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>T#114GA-C1-C5#</t>
+          <t>225-QH-D2D6-Q1214</t>
         </is>
       </c>
     </row>
@@ -499,12 +504,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>21BF-A2-LA#</t>
+          <t>114-PG-C1C5-P0105</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>T#21BF-A2-LA#</t>
+          <t>225-QH-D2D6-Q1216</t>
         </is>
       </c>
     </row>
@@ -514,12 +519,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>225-QF-D2D6-Q1212</t>
+          <t>114-S-C1C4-I0101</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>T#225-QF-D2D6-Q1212</t>
+          <t>225-T-D2D5-J1212</t>
         </is>
       </c>
     </row>
@@ -529,12 +534,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>225-QF-D2D6-Q1213</t>
+          <t>114-S-C1C4-I0102</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>T#225-QF-D2D6-Q1213</t>
+          <t>225-T-D2D5-J1213</t>
         </is>
       </c>
     </row>
@@ -544,12 +549,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>225HB-D2-D6#</t>
+          <t>114CH-C1-C5#</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>T#225HB-D2-D6#</t>
+          <t>225DI-D2-D6#</t>
         </is>
       </c>
     </row>
@@ -559,12 +564,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>27GA-C4-C5#</t>
+          <t>114GA-C1-C5#</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>T#27GA-C4-C5#</t>
+          <t>225HB-D2-D6#</t>
         </is>
       </c>
     </row>
@@ -574,12 +579,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>32CG-B3-MB#</t>
+          <t>168-S-C1B4-I0101</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>T#32CG-B3-MB#</t>
+          <t>279-T-D2C5-J1212</t>
         </is>
       </c>
     </row>
@@ -589,12 +594,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>33-FG-C2C5-P0106</t>
+          <t>168-S-C1B4-IO101</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>T#33-FG-C2C5-P0106</t>
+          <t>279-T-D2C5-JP212</t>
         </is>
       </c>
     </row>
@@ -604,12 +609,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>33GA-C4-C5</t>
+          <t>168GA-C6-C5#</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>T#33GA-C4-C5</t>
+          <t>279HB-D7-D6#</t>
         </is>
       </c>
     </row>
@@ -619,12 +624,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>33GA-C4-C5#</t>
+          <t>219-PG-C1C5-X050</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>T#33GA-C4-C5#</t>
+          <t>320-QH-D2D6-Y161</t>
         </is>
       </c>
     </row>
@@ -634,12 +639,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>44HB-D5-D6</t>
+          <t>21BF-A2-LA#</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>T#44HB-D5-D6</t>
+          <t>32CG-B3-MB#</t>
         </is>
       </c>
     </row>
@@ -649,12 +654,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>89-S-C1C5-I0104</t>
+          <t>27BR-A2-LA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>T#89-S-C1C5-I0104</t>
+          <t>38CS-B3-MB</t>
         </is>
       </c>
     </row>
@@ -664,12 +669,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>89GA-C1-C5#</t>
+          <t>27GA-C4-C5#</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>T#89GA-C1-C5#</t>
+          <t>38HB-D5-D6#</t>
         </is>
       </c>
     </row>
@@ -679,12 +684,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>90-T-D2D6-J1215</t>
+          <t>27GA-C4-L8</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>T#90-T-D2D6-J1215</t>
+          <t>38HB-D5-M9</t>
         </is>
       </c>
     </row>
@@ -694,12 +699,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AJ-Q1222</t>
+          <t>27GA-C4-L8#</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>T#AJ-Q1222</t>
+          <t>38HB-D5-M9#</t>
         </is>
       </c>
     </row>
@@ -709,12 +714,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>AJ-Q1223</t>
+          <t>324-PE-C1C5-X040</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>T#AJ-Q1223</t>
+          <t>435-QF-D2D6-Y151</t>
         </is>
       </c>
     </row>
@@ -724,12 +729,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ATD-Q1223</t>
+          <t>324-S-C1B4-X000</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>T#ATD-Q1223</t>
+          <t>435-T-D2C5-Y111</t>
         </is>
       </c>
     </row>
@@ -739,12 +744,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ATP-Q1222</t>
+          <t>33-FG-C2C5-I0107</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>T#ATP-Q1222</t>
+          <t>44-GH-D3D6-J1218</t>
         </is>
       </c>
     </row>
@@ -754,12 +759,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ATP-Q1223</t>
+          <t>33-FG-C2C5-I0108</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>T#ATP-Q1223</t>
+          <t>44-GH-D3D6-J1219</t>
         </is>
       </c>
     </row>
@@ -769,12 +774,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CLIENT LINE NUMBER</t>
+          <t>33-FG-C2C5-I0112</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>T#CLIENT LINE NUMBER</t>
+          <t>44-GH-D3D6-J1223</t>
         </is>
       </c>
     </row>
@@ -784,12 +789,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CLIENT VALVE INFO</t>
+          <t>33-FG-C2C5-P0106</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>T#CLIENT VALVE INFO</t>
+          <t>44-GH-D3D6-Q1217</t>
         </is>
       </c>
     </row>
@@ -799,12 +804,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>HS-P0116</t>
+          <t>33-FG-C2C5-P0107</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>T#HS-P0116</t>
+          <t>44-GH-D3D6-Q1218</t>
         </is>
       </c>
     </row>
@@ -814,12 +819,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>HS-XXXXX</t>
+          <t>33-IA-A2B1-I0109</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>T#HS-XXXXX</t>
+          <t>44-JB-B3C2-J1210</t>
         </is>
       </c>
     </row>
@@ -829,12 +834,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>I-P0110</t>
+          <t>33-IA-A2B1-P0108</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>T#I-P0110</t>
+          <t>44-JB-B3C2-Q1219</t>
         </is>
       </c>
     </row>
@@ -844,12 +849,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>I-P0112</t>
+          <t>33BR-A2-LA#</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>T#I-P0112</t>
+          <t>44CS-B3-MB#</t>
         </is>
       </c>
     </row>
@@ -859,12 +864,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>I-XXXXX</t>
+          <t>33CH-C3-L5#</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>T#I-XXXXX</t>
+          <t>44DI-D4-M6#</t>
         </is>
       </c>
     </row>
@@ -874,12 +879,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>IT-Q1227</t>
+          <t>33GA-A2-L8</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>T#IT-Q1227</t>
+          <t>44HB-B3-M9</t>
         </is>
       </c>
     </row>
@@ -889,12 +894,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>J-Q1223</t>
+          <t>33GA-C3-L8#</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>T#J-Q1223</t>
+          <t>44HB-D4-M9#</t>
         </is>
       </c>
     </row>
@@ -904,12 +909,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>NOTE 13</t>
+          <t>33GA-C4-C5</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>T#NOTE 13</t>
+          <t>44HB-D5-D6</t>
         </is>
       </c>
     </row>
@@ -919,12 +924,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>OPUF 24</t>
+          <t>33GA-C4-C5#</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>T#OPUF 24</t>
+          <t>44HB-D5-D6#</t>
         </is>
       </c>
     </row>
@@ -934,12 +939,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PIC-P0116</t>
+          <t>33GA-C4-L8</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>T#PIC-P0116</t>
+          <t>44HB-D5-M9</t>
         </is>
       </c>
     </row>
@@ -949,12 +954,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PIC-XXXXX</t>
+          <t>33GA-C4-L8#</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>T#PIC-XXXXX</t>
+          <t>44HB-D5-M9#</t>
         </is>
       </c>
     </row>
@@ -964,12 +969,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PT-P0116</t>
+          <t>33GL-C3-C5#</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>T#PT-P0116</t>
+          <t>44HM-D4-D6#</t>
         </is>
       </c>
     </row>
@@ -979,12 +984,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PT-XXXXX</t>
+          <t>33NE-C3-S50#</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>T#PT-XXXXX</t>
+          <t>44OF-D4-T61#</t>
         </is>
       </c>
     </row>
@@ -994,12 +999,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PV-P0110</t>
+          <t>60-FG-C1C4-I0110</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>T#PV-P0110</t>
+          <t>71-GH-D2D5-J1221</t>
         </is>
       </c>
     </row>
@@ -1009,12 +1014,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PY-P0110</t>
+          <t>60-FG-C2C5-I0106</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>T#PY-P0110</t>
+          <t>71-GH-D3D6-J1217</t>
         </is>
       </c>
     </row>
@@ -1024,12 +1029,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PY-XXXXX</t>
+          <t>60-FG-C2C5-I0110</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>T#PY-XXXXX</t>
+          <t>71-GH-D3D6-J1221</t>
         </is>
       </c>
     </row>
@@ -1039,12 +1044,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>QJD-Q1227</t>
+          <t>60-IA-A2B1-X030</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>T#QJD-Q1227</t>
+          <t>71-JB-B3C2-Y141</t>
         </is>
       </c>
     </row>
@@ -1054,12 +1059,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>QU-Q1227</t>
+          <t>60CH-C1-C5#</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>T#QU-Q1227</t>
+          <t>71DI-D2-D6#</t>
         </is>
       </c>
     </row>
@@ -1069,12 +1074,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>QZ-Q1221</t>
+          <t>60GA-C1-C5#</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>T#QZ-Q1221</t>
+          <t>71HB-D2-D6#</t>
         </is>
       </c>
     </row>
@@ -1084,12 +1089,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SAV-P0110</t>
+          <t>60GA-C1-L8#</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>T#SAV-P0110</t>
+          <t>71HB-D2-M9#</t>
         </is>
       </c>
     </row>
@@ -1099,12 +1104,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SAV-XXXXX</t>
+          <t>89-FG-C2C5-X010</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>T#SAV-XXXXX</t>
+          <t>90-GH-D3D6-Y121</t>
         </is>
       </c>
     </row>
@@ -1114,12 +1119,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>TI-P0108</t>
+          <t>89-PE-C1C5-I0105</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>T#TI-P0108</t>
+          <t>90-QF-D2D6-J1216</t>
         </is>
       </c>
     </row>
@@ -1129,12 +1134,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TO FV-P0115</t>
+          <t>89-PE-C1C5-I0111</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>T#TO FV-P0115</t>
+          <t>90-QF-D2D6-J1222</t>
         </is>
       </c>
     </row>
@@ -1144,12 +1149,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TO KV-P0113</t>
+          <t>89-PG-C1C5-P0104</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>T#TO KV-P0113</t>
+          <t>90-QH-D2D6-Q1215</t>
         </is>
       </c>
     </row>
@@ -1159,12 +1164,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TO PV-P0104</t>
+          <t>89-S-C1B4-I0102</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>T#TO PV-P0104</t>
+          <t>90-T-D2C5-J1213</t>
         </is>
       </c>
     </row>
@@ -1174,12 +1179,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TO PV-P0110</t>
+          <t>89-S-C1C4-I0103</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>T#TO PV-P0110</t>
+          <t>90-T-D2D5-J1214</t>
         </is>
       </c>
     </row>
@@ -1189,12 +1194,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>TO XV-P0105</t>
+          <t>89-S-C1C5-I0104</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>T#TO XV-P0105</t>
+          <t>90-T-D2D6-J1215</t>
         </is>
       </c>
     </row>
@@ -1204,12 +1209,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>TO XV-P0106</t>
+          <t>89CH-C1-C5#</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>T#TO XV-P0106</t>
+          <t>90DI-D2-D6#</t>
         </is>
       </c>
     </row>
@@ -1219,12 +1224,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TO XV-P0111</t>
+          <t>89GA-C1-C5</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>T#TO XV-P0111</t>
+          <t>90HB-D2-D6</t>
         </is>
       </c>
     </row>
@@ -1234,12 +1239,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>TO XV-P0112</t>
+          <t>89GA-C1-C5#</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>T#TO XV-P0112</t>
+          <t>90HB-D2-D6#</t>
         </is>
       </c>
     </row>
@@ -1249,12 +1254,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>UP GW-Q1226</t>
+          <t>FE-I0101</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>T#UP GW-Q1226</t>
+          <t>GF-J1212</t>
         </is>
       </c>
     </row>
@@ -1264,12 +1269,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>UP LW-Q1224</t>
+          <t>FE-I0103</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>T#UP LW-Q1224</t>
+          <t>GF-J1214</t>
         </is>
       </c>
     </row>
@@ -1279,12 +1284,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>UP QW-Q1215</t>
+          <t>FE-I0105</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>T#UP QW-Q1215</t>
+          <t>GF-J1216</t>
         </is>
       </c>
     </row>
@@ -1294,12 +1299,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>UP QW-Q1221</t>
+          <t>FE-P0114</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>T#UP QW-Q1221</t>
+          <t>GF-Q1225</t>
         </is>
       </c>
     </row>
@@ -1309,12 +1314,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>UP YW-Q1216</t>
+          <t>FI-I0106</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>T#UP YW-Q1216</t>
+          <t>GJ-J1217</t>
         </is>
       </c>
     </row>
@@ -1324,12 +1329,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>UP YW-Q1217</t>
+          <t>FIC-I0101</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>T#UP YW-Q1217</t>
+          <t>GJD-J1212</t>
         </is>
       </c>
     </row>
@@ -1339,12 +1344,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>UP YW-Q1222</t>
+          <t>FIC-I0103</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>T#UP YW-Q1222</t>
+          <t>GJD-J1214</t>
         </is>
       </c>
     </row>
@@ -1354,12 +1359,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>UP YW-Q1223</t>
+          <t>FIC-I0105</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>T#UP YW-Q1223</t>
+          <t>GJD-J1216</t>
         </is>
       </c>
     </row>
@@ -1369,12 +1374,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ZI-P0111</t>
+          <t>FIC-P0114</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>T#ZI-P0111</t>
+          <t>GJD-Q1225</t>
         </is>
       </c>
     </row>
@@ -1384,12 +1389,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ZI-P0112</t>
+          <t>FQI-I0105</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>T#ZI-P0112</t>
+          <t>GRJ-J1216</t>
         </is>
       </c>
     </row>
@@ -1399,12 +1404,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ZI-XXXXX</t>
+          <t>FQI-P0114</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>T#ZI-XXXXX</t>
+          <t>GRJ-Q1225</t>
         </is>
       </c>
     </row>
@@ -1414,12 +1419,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ZSC-P0112</t>
+          <t>FT-I0101</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>T#ZSC-P0112</t>
+          <t>GU-J1212</t>
         </is>
       </c>
     </row>
@@ -1429,12 +1434,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ZSC-XXXXX</t>
+          <t>FT-I0103</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>T#ZSC-XXXXX</t>
+          <t>GU-J1214</t>
         </is>
       </c>
     </row>
@@ -1444,12 +1449,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ZSO-P0111</t>
+          <t>FT-I0105</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>T#ZSO-P0111</t>
+          <t>GU-J1216</t>
         </is>
       </c>
     </row>
@@ -1459,12 +1464,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ZSO-P0112</t>
+          <t>FT-P0114</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>T#ZSO-P0112</t>
+          <t>GU-Q1225</t>
         </is>
       </c>
     </row>
@@ -1474,12 +1479,1287 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ZSO-XXXXX</t>
+          <t>FV-I0101</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>T#ZSO-XXXXX</t>
+          <t>GW-J1212</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>0</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>FV-I0103</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>GW-J1214</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>0</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>FV-I0105</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>GW-J1216</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>0</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>FV-P0115</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>GW-Q1226</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>0</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>FY-I0101</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>GZ-J1212</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>0</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>FY-I0103</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>GZ-J1214</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>0</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>FY-I0105</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>GZ-J1216</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>0</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>FY-P0115</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>GZ-Q1226</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>0</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>HS-I0102</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>IT-J1213</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>0</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>HS-I0105</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>IT-J1216</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>0</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>HS-P0116</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>IT-Q1227</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>0</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>I-I0101</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>J-J1212</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>0</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>I-I0103</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>J-J1214</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>0</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>I-I0105</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>J-J1216</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>0</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>I-P0104</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>J-Q1215</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>0</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>I-P0105</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>J-Q1216</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>0</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>I-P0106</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>J-Q1217</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>0</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>I-P0110</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>J-Q1221</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>0</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>I-P0111</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>J-Q1222</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>0</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>I-P0112</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>J-Q1223</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>0</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>I-P0113</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>J-Q1224</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>0</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>I-P0115</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>J-Q1226</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>0</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>KV-P0113</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>LW-Q1224</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>0</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>PDI-P0104</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>QEJ-Q1215</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>0</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>PIC-I0102</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>QJD-J1213</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>0</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>PIC-I0104</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>QJD-J1215</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>0</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>PIC-I0105</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>QJD-J1216</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>0</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>PIC-P0104</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>QJD-Q1215</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>0</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>PIC-P0110</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>QJD-Q1221</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>0</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>PIC-P0116</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>QJD-Q1227</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>0</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>PT-I0102</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>QU-J1213</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>0</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>PT-I0104</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>QU-J1215</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>0</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>PT-I0105</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>QU-J1216</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>0</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>PT-P0104</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>QU-Q1215</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>0</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>PT-P0110</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>QU-Q1221</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>0</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>PT-P0116</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>QU-Q1227</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>0</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>PV-P0104</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>QW-Q1215</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>0</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>PV-P0110</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>QW-Q1221</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>0</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>PY-P0104</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>QZ-Q1215</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>0</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>PY-P0110</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>QZ-Q1221</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>0</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>SAV-I0101</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>TBW-J1212</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>0</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>SAV-I0103</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>TBW-J1214</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>0</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>SAV-I0105</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>TBW-J1216</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>0</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>SAV-P0104</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>TBW-Q1215</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>0</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>SAV-P0105</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>TBW-Q1216</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>0</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>SAV-P0106</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>TBW-Q1217</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>0</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>SAV-P0110</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>TBW-Q1221</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>0</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>SAV-P0111</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>TBW-Q1222</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>0</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>SAV-P0112</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>TBW-Q1223</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>0</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>SAV-P0113</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>TBW-Q1224</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>0</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>SAV-P0115</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>TBW-Q1226</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>0</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>TI-P0102</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>UJ-Q1213</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>0</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>TI-P0108</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>UJ-Q1219</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>0</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>TO FV-IO101</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>UP GW-JP212</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>0</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>TO FV-IO103</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>UP GW-JP214</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>0</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>TO FV-IO105</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>UP GW-JP216</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>0</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>TO FV-P0115</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>UP GW-Q1226</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>0</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>TO KV-P0113</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>UP LW-Q1224</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>0</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>TO PV-P0104</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>UP QW-Q1215</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>0</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>TO PV-P0110</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>UP QW-Q1221</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>0</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>TO XV-P0105</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>UP YW-Q1216</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>0</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>TO XV-P0106</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>UP YW-Q1217</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>0</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>TO XV-P0111</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>UP YW-Q1222</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>0</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>TO XV-P0112</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>UP YW-Q1223</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>0</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>TT-P0102</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>UU-Q1213</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>0</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>TT-P0108</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>UU-Q1219</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>0</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>TW-P0102</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>UX-Q1213</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>0</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>TW-P0108</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>UX-Q1219</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>0</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>XV-P0105</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>YW-Q1216</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>0</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>XV-P0106</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>YW-Q1217</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>0</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>XV-P0111</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>YW-Q1222</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>0</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>XV-P0112</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>YW-Q1223</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>0</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>ZA-P0105</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>AB-Q1216</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>0</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>ZA-P0111</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>AB-Q1222</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>0</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>ZI-P0105</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>AJ-Q1216</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>0</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>ZI-P0106</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>AJ-Q1217</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>0</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>ZI-P0111</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>AJ-Q1222</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>0</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>ZI-P0112</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>AJ-Q1223</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>0</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>ZSC-P0105</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>ATD-Q1216</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>0</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>ZSC-P0106</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>ATD-Q1217</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>0</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>ZSC-P0111</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>ATD-Q1222</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>0</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>ZSC-P0112</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>ATD-Q1223</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>0</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>ZSO-P0105</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>ATP-Q1216</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>0</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>ZSO-P0106</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>ATP-Q1217</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>0</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>ZSO-P0111</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>ATP-Q1222</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>0</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>ZSO-P0112</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>ATP-Q1223</t>
         </is>
       </c>
     </row>

</xml_diff>